<commit_message>
Review persona projects and task answers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-science/nadia/getting-to-school.xlsx
+++ b/data-science/nadia/getting-to-school.xlsx
@@ -1792,7 +1792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MRT or LRT, with or without a bus</t>
+          <t>MRT, LRT or mixed trips</t>
         </is>
       </c>
       <c r="C3">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MRT or LRT, with or without a bus</t>
+          <t>MRT, LRT or mixed trips</t>
         </is>
       </c>
       <c r="C4">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MRT or LRT, with or without a bus</t>
+          <t>MRT, LRT or mixed trips</t>
         </is>
       </c>
       <c r="C5">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MRT or LRT, with or without a bus</t>
+          <t>MRT, LRT or mixed trips</t>
         </is>
       </c>
       <c r="C6">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MRT or LRT, with or without a bus</t>
+          <t>MRT, LRT or mixed trips</t>
         </is>
       </c>
       <c r="C12">
@@ -2398,6 +2398,7 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -2470,7 +2471,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Kept only Primary and Secondary. My P6 class is about to move from one to the other. I dropped the other six levels.</t>
+          <t>Kept only Primary and Secondary. My P6 class is about to move from one to the other. I dropped the other five levels.</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2481,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Merged 11 ways of travel into 6 groups. Groups under 1% are hard to see and add reading load. Car Only and Taxi/Private Hire Car Only became Car, taxi or private-hire car. The three rail rows became MRT or LRT, with or without a bus. Lorry/Pickup, Motorcycle/Scooter and Others became Other ways. No Transport Required became No transport needed. The Groups tab shows every row.</t>
+          <t>Merged 11 ways of travel into 6 groups. Groups under 1% are hard to see and add reading load. Car Only and Taxi/Private Hire Car Only became Car, taxi or private-hire car. The two rail rows, plus the mixed row (rail or bus with other ways), became MRT, LRT or mixed trips. Lorry/Pickup, Motorcycle/Scooter and Others became Other ways. No Transport Required became No transport needed. The Groups tab shows every row.</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2587,6 @@
       <c r="D3" t="n">
         <v>10</v>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -2628,7 +2628,6 @@
       <c r="D5" t="n">
         <v>15</v>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2647,7 +2646,6 @@
       <c r="D6" t="n">
         <v>5</v>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2666,7 +2664,6 @@
       <c r="D7" t="n">
         <v>20</v>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2685,7 +2682,6 @@
       <c r="D8" t="n">
         <v>8</v>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2727,7 +2723,6 @@
       <c r="D10" t="n">
         <v>10</v>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2769,7 +2764,6 @@
       <c r="D12" t="n">
         <v>25</v>
       </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2788,7 +2782,6 @@
       <c r="D13" t="n">
         <v>45</v>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2807,7 +2800,6 @@
       <c r="D14" t="n">
         <v>12</v>
       </c>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2846,7 +2838,6 @@
       <c r="D16" t="n">
         <v>40</v>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2857,7 +2848,6 @@
           <t>Car</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>Blank: left blank</t>
@@ -2881,7 +2871,6 @@
       <c r="D18" t="n">
         <v>7</v>
       </c>
-      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2923,7 +2912,6 @@
       <c r="D20" t="n">
         <v>20</v>
       </c>
-      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2942,7 +2930,6 @@
       <c r="D21" t="n">
         <v>10</v>
       </c>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2981,7 +2968,6 @@
       <c r="D23" t="n">
         <v>20</v>
       </c>
-      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3023,7 +3009,6 @@
       <c r="D25" t="n">
         <v>30</v>
       </c>
-      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -3042,7 +3027,6 @@
       <c r="D26" t="n">
         <v>6</v>
       </c>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3061,7 +3045,6 @@
       <c r="D27" t="n">
         <v>12</v>
       </c>
-      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3080,7 +3063,6 @@
       <c r="D28" t="n">
         <v>25</v>
       </c>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -3119,7 +3101,6 @@
       <c r="D30" t="n">
         <v>18</v>
       </c>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -3138,7 +3119,6 @@
       <c r="D31" t="n">
         <v>10</v>
       </c>
-      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -3157,7 +3137,6 @@
       <c r="D32" t="n">
         <v>15</v>
       </c>
-      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3176,183 +3155,154 @@
       <c r="D33" t="n">
         <v>5</v>
       </c>
-      <c r="E33" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="34"/>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
       <c r="B35" s="8" t="inlineStr">
         <is>
           <t>How many numbers</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
       <c r="D35">
         <f>COUNT(D3:D33)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
       <c r="B36" s="8" t="inlineStr">
         <is>
           <t>AVERAGE (mean)</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
       <c r="D36">
         <f>ROUND(AVERAGE(D3:D33),1)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr"/>
       <c r="B37" s="8" t="inlineStr">
         <is>
           <t>MEDIAN (middle)</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
       <c r="D37">
         <f>MEDIAN(D3:D33)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
       <c r="B38" s="8" t="inlineStr">
         <is>
           <t>MIN (shortest)</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
       <c r="D38">
         <f>MIN(D3:D33)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
       <c r="B39" s="8" t="inlineStr">
         <is>
           <t>MAX (longest)</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
       <c r="D39">
         <f>MAX(D3:D33)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
       <c r="B40" s="8" t="inlineStr">
         <is>
           <t>Range (longest minus shortest)</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
       <c r="D40">
         <f>MAX(D3:D33)-MIN(D3:D33)</f>
         <v/>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
       <c r="B42" s="8" t="inlineStr">
         <is>
           <t>Count by way of travel (rows with a duplicate removed)</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
           <t>Walk</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
       <c r="D43">
         <f>COUNTIFS(B3:B33,"Walk",E3:E33,"&lt;&gt;Slip 12 typed twice: not counted")</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
           <t>Car</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
       <c r="D44">
         <f>COUNTIFS(B3:B33,"Car",E3:E33,"&lt;&gt;Slip 12 typed twice: not counted")</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
           <t>School bus</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
       <c r="D45">
         <f>COUNTIFS(B3:B33,"School bus",E3:E33,"&lt;&gt;Slip 12 typed twice: not counted")</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
           <t>Public bus</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
       <c r="D46">
         <f>COUNTIFS(B3:B33,"Public bus",E3:E33,"&lt;&gt;Slip 12 typed twice: not counted")</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
           <t>MRT and bus</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
       <c r="D47">
         <f>COUNTIFS(B3:B33,"MRT and bus",E3:E33,"&lt;&gt;Slip 12 typed twice: not counted")</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
           <t>Prefer not to say</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
       <c r="D48">
         <f>COUNTIFS(B3:B33,"Prefer not to say",E3:E33,"&lt;&gt;Slip 12 typed twice: not counted")</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
           <t>Rule: before showing the class, merge any group under 5 into Other or not said.</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>